<commit_message>
Add company ıd column to reconciliation excel template
</commit_message>
<xml_diff>
--- a/wwwroot/templates/MutabakatTemplate.xlsx
+++ b/wwwroot/templates/MutabakatTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOD\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8875FF0F-A5A0-4F8C-94E2-733AF3D3FE14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E5CE01-8FF5-476C-9859-2DF4EC06E2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6960" yWindow="6900" windowWidth="16950" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5490" yWindow="4665" windowWidth="16950" windowHeight="10935" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MutabakatTemplate" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
   <si>
     <t>MutabakatId</t>
   </si>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t>MutabakatGonderimDurumu</t>
+  </si>
+  <si>
+    <t>FirmaId</t>
   </si>
 </sst>
 </file>
@@ -402,19 +405,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="27.42578125" customWidth="1"/>
-    <col min="7" max="7" width="23" customWidth="1"/>
-    <col min="8" max="8" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="27.42578125" customWidth="1"/>
+    <col min="8" max="8" width="23" customWidth="1"/>
+    <col min="9" max="9" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -422,125 +425,140 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>13</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>-4500</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2" s="1">
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" s="1">
         <v>46113</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>3000</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>11</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3" s="1">
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1">
         <v>46113</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
         <v>7</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>8500</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>11</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>2</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <v>46114</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
         <v>9</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>8275</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>11</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>2</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>46115</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove unnecessary explanation column from reconciliation excel
</commit_message>
<xml_diff>
--- a/wwwroot/templates/MutabakatTemplate.xlsx
+++ b/wwwroot/templates/MutabakatTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E5CE01-8FF5-476C-9859-2DF4EC06E2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE77927-0CBC-487E-B6BA-796988316956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5490" yWindow="4665" windowWidth="16950" windowHeight="10935" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7485" yWindow="1380" windowWidth="16950" windowHeight="10950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MutabakatTemplate" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>MutabakatId</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>A</t>
-  </si>
-  <si>
-    <t>a</t>
   </si>
   <si>
     <t>MutabakatGonderimDurumu</t>
@@ -425,7 +422,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -437,7 +434,7 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H1" t="s">
         <v>5</v>
@@ -470,9 +467,6 @@
       </c>
       <c r="H2" s="1">
         <v>46113</v>
-      </c>
-      <c r="I2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -500,9 +494,6 @@
       <c r="H3" s="1">
         <v>46113</v>
       </c>
-      <c r="I3" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -529,9 +520,6 @@
       <c r="H4" s="1">
         <v>46114</v>
       </c>
-      <c r="I4" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -557,9 +545,6 @@
       </c>
       <c r="H5" s="1">
         <v>46115</v>
-      </c>
-      <c r="I5" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improve validation, filtering, and UI with cari group and date refinements
</commit_message>
<xml_diff>
--- a/wwwroot/templates/MutabakatTemplate.xlsx
+++ b/wwwroot/templates/MutabakatTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE77927-0CBC-487E-B6BA-796988316956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8CEB5A-2A59-48B4-849C-F1FC57EF33D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7485" yWindow="1380" windowWidth="16950" windowHeight="10950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2295" yWindow="2910" windowWidth="16950" windowHeight="10950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MutabakatTemplate" sheetId="1" r:id="rId1"/>
@@ -457,7 +457,7 @@
         <v>7</v>
       </c>
       <c r="E2">
-        <v>-4500</v>
+        <v>4350</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -483,7 +483,7 @@
         <v>8</v>
       </c>
       <c r="E3">
-        <v>3000</v>
+        <v>15850</v>
       </c>
       <c r="F3" t="s">
         <v>11</v>
@@ -509,7 +509,7 @@
         <v>7</v>
       </c>
       <c r="E4">
-        <v>8500</v>
+        <v>7590</v>
       </c>
       <c r="F4" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Improve audit logging unified import/error logs with expandable UI support
</commit_message>
<xml_diff>
--- a/wwwroot/templates/MutabakatTemplate.xlsx
+++ b/wwwroot/templates/MutabakatTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E08C3859-46BF-47CE-9279-E566771753D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48DE8A4A-5A5D-4FDD-A0E1-6DDE52B16001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1890" yWindow="3660" windowWidth="16950" windowHeight="10950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3225" yWindow="2325" windowWidth="16950" windowHeight="10575" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MutabakatTemplate" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>MutabakatId</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>FirmaId</t>
-  </si>
-  <si>
-    <t>P8</t>
   </si>
 </sst>
 </file>
@@ -447,8 +444,8 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>14</v>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -538,10 +535,10 @@
         <v>9</v>
       </c>
       <c r="E5">
-        <v>8275</v>
+        <v>6000</v>
       </c>
       <c r="F5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G5">
         <v>2</v>

</xml_diff>